<commit_message>
Updated Standings, Box Scores
Standings to EOD 9/29/26, Box Scores with no stats for 9/29/26
</commit_message>
<xml_diff>
--- a/2026-2027/BoxScores/September.xlsx
+++ b/2026-2027/BoxScores/September.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\NHLStats\2026-2027\BoxScores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F1A4FC-17B3-427C-B669-44309AE626A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABDD2F0A-019D-440E-8AAD-631842571498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="1590" windowWidth="38640" windowHeight="15720" xr2:uid="{7901B5C0-98B5-4042-9E0B-86E022D78A84}"/>
+    <workbookView xWindow="-38520" yWindow="1590" windowWidth="38640" windowHeight="15720" activeTab="5" xr2:uid="{7901B5C0-98B5-4042-9E0B-86E022D78A84}"/>
   </bookViews>
   <sheets>
     <sheet name="Index" sheetId="1" r:id="rId1"/>
@@ -18,10 +18,11 @@
     <sheet name="Scores (9-29-26)" sheetId="3" r:id="rId3"/>
     <sheet name="Scores (9-30-26)" sheetId="7" r:id="rId4"/>
     <sheet name="Offense (9-29-26)" sheetId="5" r:id="rId5"/>
-    <sheet name="Rosters (Offense - 23)" sheetId="6" r:id="rId6"/>
-    <sheet name="Goalies (9-29-26)" sheetId="4" r:id="rId7"/>
-    <sheet name="Offense (9-30-26)" sheetId="8" r:id="rId8"/>
-    <sheet name="Goalies (9-30-26)" sheetId="9" r:id="rId9"/>
+    <sheet name="Sheet1" sheetId="10" r:id="rId6"/>
+    <sheet name="Rosters (Offense - 23)" sheetId="6" r:id="rId7"/>
+    <sheet name="Goalies (9-29-26)" sheetId="4" r:id="rId8"/>
+    <sheet name="Offense (9-30-26)" sheetId="8" r:id="rId9"/>
+    <sheet name="Goalies (9-30-26)" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="83">
   <si>
     <t>Winnipeg Jets</t>
   </si>
@@ -1103,6 +1104,85 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B3D5811-0E55-4FBC-944E-BE8472B1A8CE}">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" style="1"/>
+    <col min="3" max="3" width="22" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K2" s="15"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K3" s="15"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K4" s="15"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K5" s="15"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K6" s="15"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="K7" s="15"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="M1" location="'Scores (9-30-26)'!A1" display="HOME" xr:uid="{9C3259B6-E73D-47E1-8625-6AA630BAC14E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0148CC85-F753-4FD2-B9F3-A5962DDFE417}">
   <dimension ref="A1:O56"/>
@@ -1367,51 +1447,77 @@
       <c r="A3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="12"/>
+      <c r="B3" s="12">
+        <v>1</v>
+      </c>
       <c r="C3" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="12"/>
+      <c r="D3" s="12">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10">
+        <v>3</v>
+      </c>
       <c r="C4" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="10"/>
+      <c r="D4" s="10">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="10">
+        <v>0</v>
+      </c>
       <c r="C5" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="10"/>
+      <c r="D5" s="10">
+        <v>3</v>
+      </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10">
+        <v>6</v>
+      </c>
       <c r="C6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="10"/>
+      <c r="D6" s="10">
+        <v>5</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="7" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="8"/>
+      <c r="B7" s="8">
+        <v>2</v>
+      </c>
       <c r="C7" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="8"/>
+      <c r="D7" s="8">
+        <v>5</v>
+      </c>
     </row>
     <row r="8" spans="1:27" ht="15" thickTop="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
@@ -1654,6 +1760,18 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99EFED56-E735-49BE-877C-8E105DC78FC2}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40E9DF01-FCB0-4705-8E3F-A6211BAEC300}">
   <dimension ref="A1:V80"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2045,13 +2163,18 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="M54:N54"/>
-    <mergeCell ref="O1:P1"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="S1:T1"/>
-    <mergeCell ref="U1:V1"/>
-    <mergeCell ref="Q1:R1"/>
-    <mergeCell ref="M1:N1"/>
+    <mergeCell ref="K54:L54"/>
+    <mergeCell ref="O54:P54"/>
+    <mergeCell ref="Q54:R54"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="G28:H28"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="E54:F54"/>
+    <mergeCell ref="G54:H54"/>
+    <mergeCell ref="I54:J54"/>
     <mergeCell ref="I28:J28"/>
     <mergeCell ref="K28:L28"/>
     <mergeCell ref="M28:N28"/>
@@ -2061,29 +2184,24 @@
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="K1:L1"/>
+    <mergeCell ref="M54:N54"/>
+    <mergeCell ref="O1:P1"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="S1:T1"/>
+    <mergeCell ref="U1:V1"/>
+    <mergeCell ref="Q1:R1"/>
+    <mergeCell ref="M1:N1"/>
     <mergeCell ref="S54:T54"/>
     <mergeCell ref="S28:T28"/>
     <mergeCell ref="U28:V28"/>
     <mergeCell ref="Q28:R28"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="E54:F54"/>
-    <mergeCell ref="G54:H54"/>
-    <mergeCell ref="I54:J54"/>
-    <mergeCell ref="K54:L54"/>
-    <mergeCell ref="O54:P54"/>
-    <mergeCell ref="Q54:R54"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="G28:H28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BAF5206-6C7C-473B-8F0B-07B9A3759B8D}">
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2162,7 +2280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2152161-5074-48C0-BC51-02F90EED5F64}">
   <dimension ref="A1:U1"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2247,83 +2365,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B3D5811-0E55-4FBC-944E-BE8472B1A8CE}">
-  <dimension ref="A1:M7"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.109375" style="1"/>
-    <col min="3" max="3" width="22" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K2" s="15"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K3" s="15"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K4" s="15"/>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K5" s="15"/>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K6" s="15"/>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K7" s="15"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="M1" location="'Scores (9-30-26)'!A1" display="HOME" xr:uid="{9C3259B6-E73D-47E1-8625-6AA630BAC14E}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>